<commit_message>
[Fix] ScoringInfo - Index - 修正Export Excel 範本
</commit_message>
<xml_diff>
--- a/Platform/Platform.WebSite/ModuleResources/Other/SPA_ScoringInfo/供應商SPA評鑑計分資料匯出範本.xlsx
+++ b/Platform/Platform.WebSite/ModuleResources/Other/SPA_ScoringInfo/供應商SPA評鑑計分資料匯出範本.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\加鑫科技\1.1 客戶報價單\新竹_TET\供應商平台&amp;評鑑\系統開發\Dev(供應商評鑑_開發)\Platform\Platform.WebSite\ModuleResources\Other\SPA_ScoringInfo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\加鑫科技\1.1 客戶報價單\新竹_TET\供應商平台&amp;評鑑\系統開發\Dev(供應商平台&amp;評鑑_開發)\Platform\Platform.WebSite\ModuleResources\Other\SPA_ScoringInfo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1126DFA-97FB-448D-9262-FD756D009F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D08A5D-B5AC-4119-B297-BF13D8B35625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2984F46C-2D94-4B4A-AD03-55CBAB69B2C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{2984F46C-2D94-4B4A-AD03-55CBAB69B2C2}"/>
   </bookViews>
   <sheets>
     <sheet name="計分資料主檔" sheetId="7" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="41">
   <si>
     <t xml:space="preserve">評鑑期間 </t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -772,16 +772,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF95FE55-2604-4252-ACB4-E76A09C0D78B}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="15.77734375" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="15.77734375" customWidth="1"/>
-    <col min="10" max="10" width="25.77734375" customWidth="1"/>
+    <col min="1" max="8" width="15.77734375" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" customWidth="1"/>
+    <col min="11" max="11" width="25.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -798,18 +798,21 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>